<commit_message>
Consolida influenciadores e leads automotivos
</commit_message>
<xml_diff>
--- a/formacao/atividades-feitas/50-leads-comentarios-instagram-patagon-ai.xlsx
+++ b/formacao/atividades-feitas/50-leads-comentarios-instagram-patagon-ai.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R770a7adec4ad4a90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads 50" sheetId="2" r:id="R6e6eeed480b54284"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estratégia" sheetId="3" r:id="R147675c7baad4488"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R409ab121ae874fef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads 50" sheetId="2" r:id="R3cd0a5cdaa68417a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Estratégia" sheetId="3" r:id="Rfc380625db154fea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pesquisa pública" sheetId="4" r:id="Rbee97b0e876741d2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,7 +20,7 @@
     <x:numFmt numFmtId="200" formatCode="#,##0"/>
     <x:numFmt numFmtId="201" formatCode="dd/mm/yyyy"/>
   </x:numFmts>
-  <x:fonts count="12">
+  <x:fonts count="15">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -86,8 +87,25 @@
       <x:color rgb="FF333333"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FF15233F"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF666666"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF222222"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -124,8 +142,13 @@
         <x:fgColor rgb="FFDDEBF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF15233F"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="11">
+  <x:borders count="20">
     <x:border>
       <x:left/>
       <x:right/>
@@ -237,11 +260,122 @@
       </x:bottom>
       <x:diagonal/>
     </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:right>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:right>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:left>
+      <x:right/>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:left>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:top>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:top>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:left>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFD9DDE5"/>
+      </x:top>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="65">
+  <x:cellXfs count="85">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -373,6 +507,56 @@
     <x:xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -384,7 +568,7 @@
         <x:color rgb="FF2F6B2F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -395,7 +579,7 @@
         <x:color rgb="FF806000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -406,7 +590,7 @@
         <x:color rgb="FF9C3A18"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -417,7 +601,7 @@
         <x:color rgb="FF2F6B2F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -456,6 +640,23 @@
     <x:tableColumn id="25" name="Status da prospecção"/>
     <x:tableColumn id="26" name="Contatos na mesma conta"/>
     <x:tableColumn id="27" name="Recomendação por conta"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PublicAccountResearch" displayName="PublicAccountResearch" ref="A4:I19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="Rank"/>
+    <x:tableColumn id="2" name="Pessoa"/>
+    <x:tableColumn id="3" name="Empresa indicada"/>
+    <x:tableColumn id="4" name="Domínio/site público"/>
+    <x:tableColumn id="5" name="Confirmação pessoa–empresa"/>
+    <x:tableColumn id="6" name="Cargo/atuação em fonte pública"/>
+    <x:tableColumn id="7" name="Fontes públicas"/>
+    <x:tableColumn id="8" name="Leitura ICP / pendência"/>
+    <x:tableColumn id="9" name="Data Stone"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -5713,7 +5914,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebc183e79b69415f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89619b8034534616"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -6151,4 +6352,537 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="33" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="33" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="52" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="43" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="55" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="54" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="27" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="65" t="str">
+        <x:v>Pesquisa pública dos primeiros 15 contatos</x:v>
+      </x:c>
+      <x:c r="B1" s="65"/>
+      <x:c r="C1" s="65"/>
+      <x:c r="D1" s="65"/>
+      <x:c r="E1" s="65"/>
+      <x:c r="F1" s="65"/>
+      <x:c r="G1" s="65"/>
+      <x:c r="H1" s="65"/>
+      <x:c r="I1" s="65"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="67" t="str">
+        <x:v>Pré-validação de pessoa e conta. Fontes públicas não substituem confirmação de vínculo atual, CNPJ, porte, mídia e volume de leads. Consultas Data Stone pendentes da rotação da chave.</x:v>
+      </x:c>
+      <x:c r="B2" s="67"/>
+      <x:c r="C2" s="67"/>
+      <x:c r="D2" s="67"/>
+      <x:c r="E2" s="67"/>
+      <x:c r="F2" s="67"/>
+      <x:c r="G2" s="67"/>
+      <x:c r="H2" s="67"/>
+      <x:c r="I2" s="67"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="76" t="str">
+        <x:v>Rank</x:v>
+      </x:c>
+      <x:c r="B4" s="77" t="str">
+        <x:v>Pessoa</x:v>
+      </x:c>
+      <x:c r="C4" s="77" t="str">
+        <x:v>Empresa indicada</x:v>
+      </x:c>
+      <x:c r="D4" s="77" t="str">
+        <x:v>Domínio/site público</x:v>
+      </x:c>
+      <x:c r="E4" s="77" t="str">
+        <x:v>Confirmação pessoa–empresa</x:v>
+      </x:c>
+      <x:c r="F4" s="77" t="str">
+        <x:v>Cargo/atuação em fonte pública</x:v>
+      </x:c>
+      <x:c r="G4" s="77" t="str">
+        <x:v>Fontes públicas</x:v>
+      </x:c>
+      <x:c r="H4" s="77" t="str">
+        <x:v>Leitura ICP / pendência</x:v>
+      </x:c>
+      <x:c r="I4" s="78" t="str">
+        <x:v>Data Stone</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="79" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B5" s="80" t="str">
+        <x:v>Thiago Pinho</x:v>
+      </x:c>
+      <x:c r="C5" s="80" t="str">
+        <x:v>Pinho Concessionária de Seminovos / Grupo S Pinho</x:v>
+      </x:c>
+      <x:c r="D5" s="80" t="str">
+        <x:v>pinhoveiculos.com (link da bio; domínio/CNPJ da entidade ainda não confirmado)</x:v>
+      </x:c>
+      <x:c r="E5" s="80" t="str">
+        <x:v>Bio do Instagram associa o perfil à Pinho; há possível conflito com Pinho Chevrolet e outras empresas Pinho. Não vincular sem confirmar a entidade correta.</x:v>
+      </x:c>
+      <x:c r="F5" s="80" t="str">
+        <x:v>Empresário/presidente (autodescrição no Instagram)</x:v>
+      </x:c>
+      <x:c r="G5" s="80" t="str">
+        <x:v>https://www.instagram.com/thiagopinhotiti
+https://www.pinhoveiculos.com/</x:v>
+      </x:c>
+      <x:c r="H5" s="80" t="str">
+        <x:v>Confirmar razão social, marca/franquia e unidades. Evidência insuficiente para validar ICP.</x:v>
+      </x:c>
+      <x:c r="I5" s="81" t="str">
+        <x:v>Aguardando nova chave</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="79" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B6" s="80" t="str">
+        <x:v>Eltton Andradee</x:v>
+      </x:c>
+      <x:c r="C6" s="80" t="str">
+        <x:v>TAG Veículos</x:v>
+      </x:c>
+      <x:c r="D6" s="80" t="str">
+        <x:v>https://tagveiculosdf.com.br/</x:v>
+      </x:c>
+      <x:c r="E6" s="80" t="str">
+        <x:v>A bio do Instagram marca @tagveiculos; não localizei uma fonte profissional independente que confirme cargo atual.</x:v>
+      </x:c>
+      <x:c r="F6" s="80" t="str">
+        <x:v>Empresário (bio do Instagram)</x:v>
+      </x:c>
+      <x:c r="G6" s="80" t="str">
+        <x:v>https://www.instagram.com/elttonandradee
+https://tagveiculosdf.com.br/</x:v>
+      </x:c>
+      <x:c r="H6" s="80" t="str">
+        <x:v>Sinais públicos apontam para revenda multimarcas e operação local; provável fora do ICP de concessionária mono/multimarcas autorizada com &gt;3 unidades. Confirmar porte antes de descartar.</x:v>
+      </x:c>
+      <x:c r="I6" s="81" t="str">
+        <x:v>Aguardando nova chave</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="79" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B7" s="80" t="str">
+        <x:v>Sandra Carvalho</x:v>
+      </x:c>
+      <x:c r="C7" s="80" t="str">
+        <x:v>AK Auto Center</x:v>
+      </x:c>
+      <x:c r="D7" s="80" t="str">
+        <x:v>https://akautocenter.com.br/</x:v>
+      </x:c>
+      <x:c r="E7" s="80" t="str">
+        <x:v>Matéria da Exame a identifica como sócia-proprietária da oficina AK Auto Center.</x:v>
+      </x:c>
+      <x:c r="F7" s="80" t="str">
+        <x:v>Sócia-proprietária; gestão de oficina (Exame)</x:v>
+      </x:c>
+      <x:c r="G7" s="80" t="str">
+        <x:v>https://exame.com/negocios/empreendedoras-superam-barreiras-fazem-sucesso-mercados-masculinos/
+https://akautocenter.com.br/</x:v>
+      </x:c>
+      <x:c r="H7" s="80" t="str">
+        <x:v>A empresa aparece como oficina/reparação, não como grupo de concessionárias de marca; desqualificador provável no ICP atual.</x:v>
+      </x:c>
+      <x:c r="I7" s="81" t="str">
+        <x:v>Aguardando nova chave</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="79" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B8" s="80" t="str">
+        <x:v>Jaime Campelo Bessa</x:v>
+      </x:c>
+      <x:c r="C8" s="80" t="str">
+        <x:v>Pro Veículos Manaus / Alugue na Pro / ALVEAM</x:v>
+      </x:c>
+      <x:c r="D8" s="80" t="str">
+        <x:v>https://proveiculosmanaus.com.br/</x:v>
+      </x:c>
+      <x:c r="E8" s="80" t="str">
+        <x:v>Instagram associa o perfil às marcas; ALVEAM lista Jaime Campelo Bessa Neto, mas isso não comprova vínculo empregatício/societário com a Pro Veículos.</x:v>
+      </x:c>
+      <x:c r="F8" s="80" t="str">
+        <x:v>Atuação no mercado automotivo; cargo empresarial atual não confirmado</x:v>
+      </x:c>
+      <x:c r="G8" s="80" t="str">
+        <x:v>https://www.instagram.com/jaimedapro
+https://www.alveam.com.br/Quemsomos/
+https://proveiculosmanaus.com.br/</x:v>
+      </x:c>
+      <x:c r="H8" s="80" t="str">
+        <x:v>Site apresenta operação de veículos novos/usados em Manaus; unidade e foco de marca parecem não cumprir ICP. Verificar somente após confirmar entidade e operação.</x:v>
+      </x:c>
+      <x:c r="I8" s="81" t="str">
+        <x:v>Aguardando nova chave</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="79" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B9" s="80" t="str">
+        <x:v>Dallyane Barbosa Costa</x:v>
+      </x:c>
+      <x:c r="C9" s="80" t="str">
+        <x:v>Alagoas Motos</x:v>
+      </x:c>
+      <x:c r="D9" s="80" t="str">
+        <x:v>https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="E9" s="80" t="str">
+        <x:v>LinkedIn associa o perfil a Alagoas Motos, mas a atividade pública também menciona encerramento de ciclo; vínculo atual pode estar desatualizado.</x:v>
+      </x:c>
+      <x:c r="F9" s="80" t="str">
+        <x:v>Perfil público ligado a Web/F&amp;I; cargo e situação atuais precisam de confirmação</x:v>
+      </x:c>
+      <x:c r="G9" s="80" t="str">
+        <x:v>https://br.linkedin.com/in/dallyane-barbosa-costa-32b444184
+https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="H9" s="80" t="str">
+        <x:v>Empresa representa Honda e divulga múltiplas unidades; confirmar vínculo atual, volume WhatsApp e Ads.</x:v>
+      </x:c>
+      <x:c r="I9" s="81" t="str">
+        <x:v>Aguardando nova chave</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="79" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B10" s="80" t="str">
+        <x:v>Deyvid Bezerra</x:v>
+      </x:c>
+      <x:c r="C10" s="80" t="str">
+        <x:v>Alagoas Motos</x:v>
+      </x:c>
+      <x:c r="D10" s="80" t="str">
+        <x:v>https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="E10" s="80" t="str">
+        <x:v>Bio do Instagram indica Alagoas Motos/Honda; não encontrei confirmação profissional independente nesta rodada.</x:v>
+      </x:c>
+      <x:c r="F10" s="80" t="str">
+        <x:v>Coordenador de Vendas (bio do Instagram)</x:v>
+      </x:c>
+      <x:c r="G10" s="80" t="str">
+        <x:v>https://www.instagram.com/deyvid.honda
+https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="H10" s="80" t="str">
+        <x:v>Conta potencialmente aderente por marca/unidades; confirmar cargo atual, volume de leads e operação de mídia.</x:v>
+      </x:c>
+      <x:c r="I10" s="81" t="str">
+        <x:v>Aguardando nova chave</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="79" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B11" s="80" t="str">
+        <x:v>Emerson Angelino Cavalcante</x:v>
+      </x:c>
+      <x:c r="C11" s="80" t="str">
+        <x:v>Alagoas Motos</x:v>
+      </x:c>
+      <x:c r="D11" s="80" t="str">
+        <x:v>https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="E11" s="80" t="str">
+        <x:v>Bio do Instagram indica Alagoas Motos/Honda; não encontrei confirmação profissional independente nesta rodada.</x:v>
+      </x:c>
+      <x:c r="F11" s="80" t="str">
+        <x:v>Gerente de Consórcio / instrutor (bio do Instagram)</x:v>
+      </x:c>
+      <x:c r="G11" s="80" t="str">
+        <x:v>https://www.instagram.com/emerson.honda
+https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="H11" s="80" t="str">
+        <x:v>Confirmar se influencia atendimento de leads novos no WhatsApp e se possui escopo de decisão comercial.</x:v>
+      </x:c>
+      <x:c r="I11" s="81" t="str">
+        <x:v>Aguardando nova chave</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="79" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B12" s="80" t="str">
+        <x:v>Jefferson Furstenau</x:v>
+      </x:c>
+      <x:c r="C12" s="80" t="str">
+        <x:v>Kia Sun Motors / Suzuki Sun Motors</x:v>
+      </x:c>
+      <x:c r="D12" s="80" t="str">
+        <x:v>https://kiasunmotors.com.br/</x:v>
+      </x:c>
+      <x:c r="E12" s="80" t="str">
+        <x:v>LinkedIn identifica Kia Sun Motors como experiência/empresa do perfil.</x:v>
+      </x:c>
+      <x:c r="F12" s="80" t="str">
+        <x:v>Profissional do setor; cargo atual não ficou claro no trecho público consultado</x:v>
+      </x:c>
+      <x:c r="G12" s="80" t="str">
+        <x:v>https://br.linkedin.com/in/jefferson-furstenau-22b6a9b8
+https://kiasunmotors.com.br/</x:v>
+      </x:c>
+      <x:c r="H12" s="80" t="str">
+        <x:v>Correspondência empresa–pessoa forte; confirmar qual CNPJ/unidade e se há mais de três pontos de venda.</x:v>
+      </x:c>
+      <x:c r="I12" s="81" t="str">
+        <x:v>Aguardando nova chave</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="79" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B13" s="80" t="str">
+        <x:v>Bruno Bettéro</x:v>
+      </x:c>
+      <x:c r="C13" s="80" t="str">
+        <x:v>Alagoas Motos</x:v>
+      </x:c>
+      <x:c r="D13" s="80" t="str">
+        <x:v>https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="E13" s="80" t="str">
+        <x:v>LinkedIn associa o perfil a Alagoas Motos; Prefeitura de Arapiraca o chamou de gerente de concessionária em 2016.</x:v>
+      </x:c>
+      <x:c r="F13" s="80" t="str">
+        <x:v>Profissional/gerente de concessionária; experiência &gt;20 anos (LinkedIn)</x:v>
+      </x:c>
+      <x:c r="G13" s="80" t="str">
+        <x:v>https://br.linkedin.com/in/bruno-bett%C3%A9ro
+https://web.arapiraca.al.gov.br/2016/03/arapiraca-esta-na-contramao-da-crise-brasileira-destaca-diretor-da-honda-na-america-latina/
+https://alagoasmotos.com.br/</x:v>
+      </x:c>
+      <x:c r="H13" s="80" t="str">
+        <x:v>Corrigir empresa indicada na planilha: há evidência pública de vínculo com Alagoas Motos. Cargo atual a confirmar.</x:v>
+      </x:c>
+      <x:c r="I13" s="81" t="str">
+        <x:v>Aguardando nova chave</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="79" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B14" s="80" t="str">
+        <x:v>Gesivam Lopes</x:v>
+      </x:c>
+      <x:c r="C14" s="80" t="str">
+        <x:v>Grupo Primavia / Primavia Fiat</x:v>
+      </x:c>
+      <x:c r="D14" s="80" t="str">
+        <x:v>https://www.grupoprimavia.com.br/</x:v>
+      </x:c>
+      <x:c r="E14" s="80" t="str">
+        <x:v>LinkedIn indica Grupo Primavia; site oficial confirma grupo de concessionárias em 13 cidades e diversas marcas.</x:v>
+      </x:c>
+      <x:c r="F14" s="80" t="str">
+        <x:v>Gerente de Vendas (Instagram); vínculo com Grupo Primavia corroborado no LinkedIn</x:v>
+      </x:c>
+      <x:c r="G14" s="80" t="str">
+        <x:v>https://br.linkedin.com/in/gesivam-lopes-334512bb
+https://www.grupoprimavia.com.br/</x:v>
+      </x:c>
+      <x:c r="H14" s="80" t="str">
+        <x:v>Forte aderência de conta: grupo multiunidade e multimarcas. Confirmar unidade/brand, leads WhatsApp e Ads.</x:v>
+      </x:c>
+      <x:c r="I14" s="81" t="str">
+        <x:v>Aguardando nova chave</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="79" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B15" s="80" t="str">
+        <x:v>Keyanny</x:v>
+      </x:c>
+      <x:c r="C15" s="80" t="str">
+        <x:v>Original Yamaha</x:v>
+      </x:c>
+      <x:c r="D15" s="80" t="str">
+        <x:v>Pendente: confirmar site oficial e entidade da rede</x:v>
+      </x:c>
+      <x:c r="E15" s="80" t="str">
+        <x:v>A bio/handle Instagram indicam Yamaha Original; não encontrei correspondência profissional independente nesta rodada.</x:v>
+      </x:c>
+      <x:c r="F15" s="80" t="str">
+        <x:v>Gerente (Instagram; sem confirmação independente)</x:v>
+      </x:c>
+      <x:c r="G15" s="80" t="str">
+        <x:v>https://www.instagram.com/keyannyalves
+https://linktr.ee/yamahamotosoriginal</x:v>
+      </x:c>
+      <x:c r="H15" s="80" t="str">
+        <x:v>Confirmar razão social, domínio, vínculo e nº de unidades antes da qualificação.</x:v>
+      </x:c>
+      <x:c r="I15" s="81" t="str">
+        <x:v>Aguardando nova chave</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="79" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B16" s="80" t="str">
+        <x:v>Reinaldo R. Cardoso</x:v>
+      </x:c>
+      <x:c r="C16" s="80" t="str">
+        <x:v>Empresa não identificada</x:v>
+      </x:c>
+      <x:c r="D16" s="80" t="str">
+        <x:v>Pendente: empresa/domínio não identificados</x:v>
+      </x:c>
+      <x:c r="E16" s="80" t="str">
+        <x:v>O perfil de conteúdo automotivo e o cargo regional não bastam para associar a uma empresa específica.</x:v>
+      </x:c>
+      <x:c r="F16" s="80" t="str">
+        <x:v>Gerente Regional de Vendas (Instagram; empresa não confirmada)</x:v>
+      </x:c>
+      <x:c r="G16" s="80" t="str">
+        <x:v>https://www.instagram.com/reicardoso</x:v>
+      </x:c>
+      <x:c r="H16" s="80" t="str">
+        <x:v>Não iniciar consulta por domínio até identificar empresa atual.</x:v>
+      </x:c>
+      <x:c r="I16" s="81" t="str">
+        <x:v>Aguardando identificação da empresa</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="79" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B17" s="80" t="str">
+        <x:v>Junior Mendes</x:v>
+      </x:c>
+      <x:c r="C17" s="80" t="str">
+        <x:v>Original São Luís</x:v>
+      </x:c>
+      <x:c r="D17" s="80" t="str">
+        <x:v>https://www.originalautos.com.br/</x:v>
+      </x:c>
+      <x:c r="E17" s="80" t="str">
+        <x:v>Instagram indica Original São Luís; o domínio corresponde à rede Original consultada, mas não localizei confirmação independente desse perfil específico.</x:v>
+      </x:c>
+      <x:c r="F17" s="80" t="str">
+        <x:v>Gerente Comercial (Instagram; não corroborado por fonte profissional independente)</x:v>
+      </x:c>
+      <x:c r="G17" s="80" t="str">
+        <x:v>https://www.instagram.com/juniormendes___
+https://www.originalautos.com.br/</x:v>
+      </x:c>
+      <x:c r="H17" s="80" t="str">
+        <x:v>Conta multiunidade/multimarcas em São Luís; confirmar grupo/CNPJ e vínculo do contato.</x:v>
+      </x:c>
+      <x:c r="I17" s="81" t="str">
+        <x:v>Aguardando nova chave</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="79" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B18" s="80" t="str">
+        <x:v>Ana Angélica Omena</x:v>
+      </x:c>
+      <x:c r="C18" s="80" t="str">
+        <x:v>Grupo Gama</x:v>
+      </x:c>
+      <x:c r="D18" s="80" t="str">
+        <x:v>https://www.grupogama.com.br/</x:v>
+      </x:c>
+      <x:c r="E18" s="80" t="str">
+        <x:v>LinkedIn confirma Grupo Gama; há divergência com o cargo de Gerente Comercial atribuído na lista original.</x:v>
+      </x:c>
+      <x:c r="F18" s="80" t="str">
+        <x:v>Gerente de Qualidade, CX e Processos ligados às montadoras (LinkedIn)</x:v>
+      </x:c>
+      <x:c r="G18" s="80" t="str">
+        <x:v>https://br.linkedin.com/in/ana-ang%C3%A9lica-omena-7026327b
+https://www.grupogama.com.br/concessionarias-do-grupo</x:v>
+      </x:c>
+      <x:c r="H18" s="80" t="str">
+        <x:v>Grupo multiunidade e multimarcas. Reavaliar fit da pessoa para decisão de vendas/WhatsApp; pode ser champion de CX/processos.</x:v>
+      </x:c>
+      <x:c r="I18" s="81" t="str">
+        <x:v>Aguardando nova chave</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="82" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B19" s="83" t="str">
+        <x:v>Gessiane Nina</x:v>
+      </x:c>
+      <x:c r="C19" s="83" t="str">
+        <x:v>CAOA Chery Original São Luís</x:v>
+      </x:c>
+      <x:c r="D19" s="83" t="str">
+        <x:v>https://www.originalcaoachery.com.br/</x:v>
+      </x:c>
+      <x:c r="E19" s="83" t="str">
+        <x:v>Perfil do Instagram nomeia CAOA Chery Original; site da empresa confirma loja da Original CAOA Chery em São Luís, sem confirmar o vínculo pessoal.</x:v>
+      </x:c>
+      <x:c r="F19" s="83" t="str">
+        <x:v>Gerente Comercial (Instagram; não corroborado independentemente)</x:v>
+      </x:c>
+      <x:c r="G19" s="83" t="str">
+        <x:v>https://www.instagram.com/gessiane.nina
+https://www.originalcaoachery.com.br/empresa/nossa-historia</x:v>
+      </x:c>
+      <x:c r="H19" s="83" t="str">
+        <x:v>Conta aparentemente parte de rede maior; confirmar grupo/CNPJ, vínculo atual e escopo sobre leads.</x:v>
+      </x:c>
+      <x:c r="I19" s="84" t="str">
+        <x:v>Aguardando nova chave</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:I1"/>
+    <x:mergeCell ref="A2:I2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb11c63f365f74908"/>
+  </x:tableParts>
+</x:worksheet>
 </file>
</xml_diff>